<commit_message>
Change Cases.xlsx and Check.xlsx
</commit_message>
<xml_diff>
--- a/Cases.xlsx
+++ b/Cases.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="588" uniqueCount="302">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="593" uniqueCount="305">
   <si>
     <t>ID</t>
   </si>
@@ -747,10 +747,13 @@
     <t>TC027</t>
   </si>
   <si>
-    <t>Переход на страницу About</t>
+    <t>Переход на страницу About (проверка элементов)</t>
   </si>
   <si>
     <t>1. Меню открывается, кнопка About активна</t>
+  </si>
+  <si>
+    <t>2. Пользователь переходит на страницу About - видна версия, Privacy Policy, Terms of Use</t>
   </si>
   <si>
     <t>TC028</t>
@@ -790,6 +793,9 @@
     <t>1. Приложение работает и не падает</t>
   </si>
   <si>
+    <t>Пропущен. Проверяется в рамках smoke теста вручную</t>
+  </si>
+  <si>
     <t>2. Отключить мобильные данные</t>
   </si>
   <si>
@@ -862,6 +868,9 @@
   </si>
   <si>
     <t>1. Календарь отображается</t>
+  </si>
+  <si>
+    <t>Пропущен как Low-приоритетный. Проверяется в рамках smoke теста вручную</t>
   </si>
   <si>
     <t>2. Попытаться выбрать вчерашнюю дату</t>
@@ -1174,7 +1183,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="28">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1249,8 +1258,6 @@
     <xf borderId="2" fillId="9" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
@@ -3131,7 +3138,9 @@
       <c r="G97" s="11" t="s">
         <v>188</v>
       </c>
-      <c r="H97" s="26"/>
+      <c r="H97" s="12" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="14"/>
@@ -3169,7 +3178,9 @@
       <c r="G99" s="11" t="s">
         <v>195</v>
       </c>
-      <c r="H99" s="26"/>
+      <c r="H99" s="12" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="14"/>
@@ -3207,7 +3218,9 @@
       <c r="G101" s="11" t="s">
         <v>202</v>
       </c>
-      <c r="H101" s="26"/>
+      <c r="H101" s="12" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="14"/>
@@ -3245,7 +3258,9 @@
       <c r="G103" s="11" t="s">
         <v>206</v>
       </c>
-      <c r="H103" s="26"/>
+      <c r="H103" s="12" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="14"/>
@@ -3257,16 +3272,16 @@
         <v>45</v>
       </c>
       <c r="G104" s="11" t="s">
-        <v>46</v>
+        <v>207</v>
       </c>
       <c r="H104" s="14"/>
     </row>
     <row r="105">
       <c r="A105" s="18" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B105" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C105" s="19" t="s">
         <v>10</v>
@@ -3275,22 +3290,24 @@
         <v>25</v>
       </c>
       <c r="E105" s="18" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="F105" s="11" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="G105" s="11" t="s">
-        <v>211</v>
-      </c>
-      <c r="H105" s="27"/>
+        <v>212</v>
+      </c>
+      <c r="H105" s="21" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="18" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B106" s="18" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C106" s="19" t="s">
         <v>10</v>
@@ -3299,22 +3316,24 @@
         <v>25</v>
       </c>
       <c r="E106" s="18" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="F106" s="11" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="G106" s="11" t="s">
-        <v>211</v>
-      </c>
-      <c r="H106" s="27"/>
+        <v>212</v>
+      </c>
+      <c r="H106" s="21" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="8" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B107" s="8" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C107" s="9" t="s">
         <v>10</v>
@@ -3323,15 +3342,17 @@
         <v>25</v>
       </c>
       <c r="E107" s="8" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="F107" s="11" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="G107" s="11" t="s">
-        <v>218</v>
-      </c>
-      <c r="H107" s="26"/>
+        <v>219</v>
+      </c>
+      <c r="H107" s="22" t="s">
+        <v>220</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="13"/>
@@ -3340,10 +3361,10 @@
       <c r="D108" s="13"/>
       <c r="E108" s="13"/>
       <c r="F108" s="11" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="G108" s="11" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="H108" s="13"/>
     </row>
@@ -3354,19 +3375,19 @@
       <c r="D109" s="14"/>
       <c r="E109" s="14"/>
       <c r="F109" s="11" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="G109" s="11" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="H109" s="14"/>
     </row>
     <row r="110">
       <c r="A110" s="8" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B110" s="8" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="C110" s="9" t="s">
         <v>10</v>
@@ -3375,15 +3396,17 @@
         <v>25</v>
       </c>
       <c r="E110" s="8" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="F110" s="11" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="G110" s="11" t="s">
-        <v>218</v>
-      </c>
-      <c r="H110" s="26"/>
+        <v>219</v>
+      </c>
+      <c r="H110" s="22" t="s">
+        <v>220</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="13"/>
@@ -3392,10 +3415,10 @@
       <c r="D111" s="13"/>
       <c r="E111" s="13"/>
       <c r="F111" s="11" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="G111" s="11" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="H111" s="13"/>
     </row>
@@ -3406,19 +3429,19 @@
       <c r="D112" s="14"/>
       <c r="E112" s="14"/>
       <c r="F112" s="11" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="G112" s="11" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="H112" s="14"/>
     </row>
     <row r="113">
       <c r="A113" s="8" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B113" s="8" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="C113" s="9" t="s">
         <v>10</v>
@@ -3427,15 +3450,17 @@
         <v>25</v>
       </c>
       <c r="E113" s="8" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="F113" s="11" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="G113" s="11" t="s">
-        <v>218</v>
-      </c>
-      <c r="H113" s="26"/>
+        <v>219</v>
+      </c>
+      <c r="H113" s="22" t="s">
+        <v>220</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="13"/>
@@ -3444,10 +3469,10 @@
       <c r="D114" s="13"/>
       <c r="E114" s="13"/>
       <c r="F114" s="11" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="G114" s="11" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="H114" s="13"/>
     </row>
@@ -3461,7 +3486,7 @@
         <v>51</v>
       </c>
       <c r="G115" s="11" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="H115" s="13"/>
     </row>
@@ -3472,19 +3497,19 @@
       <c r="D116" s="14"/>
       <c r="E116" s="14"/>
       <c r="F116" s="11" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="G116" s="11" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="H116" s="14"/>
     </row>
     <row r="117">
       <c r="A117" s="8" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B117" s="8" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="C117" s="9" t="s">
         <v>10</v>
@@ -3493,15 +3518,17 @@
         <v>25</v>
       </c>
       <c r="E117" s="8" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="F117" s="11" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="G117" s="11" t="s">
-        <v>218</v>
-      </c>
-      <c r="H117" s="26"/>
+        <v>219</v>
+      </c>
+      <c r="H117" s="22" t="s">
+        <v>220</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="13"/>
@@ -3510,10 +3537,10 @@
       <c r="D118" s="13"/>
       <c r="E118" s="13"/>
       <c r="F118" s="11" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="G118" s="11" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="H118" s="13"/>
     </row>
@@ -3527,7 +3554,7 @@
         <v>51</v>
       </c>
       <c r="G119" s="11" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="H119" s="13"/>
     </row>
@@ -3538,19 +3565,19 @@
       <c r="D120" s="14"/>
       <c r="E120" s="14"/>
       <c r="F120" s="11" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="G120" s="11" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="H120" s="14"/>
     </row>
     <row r="121">
       <c r="A121" s="25" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B121" s="8" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="C121" s="9" t="s">
         <v>10</v>
@@ -3559,36 +3586,38 @@
         <v>62</v>
       </c>
       <c r="E121" s="8" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="F121" s="16" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="G121" s="16" t="s">
-        <v>242</v>
-      </c>
-      <c r="H121" s="26"/>
-    </row>
-    <row r="122">
+        <v>244</v>
+      </c>
+      <c r="H121" s="22" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="122" ht="108.0" customHeight="1">
       <c r="A122" s="14"/>
       <c r="B122" s="14"/>
       <c r="C122" s="14"/>
       <c r="D122" s="14"/>
       <c r="E122" s="14"/>
       <c r="F122" s="16" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="G122" s="16" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="H122" s="14"/>
     </row>
     <row r="123">
       <c r="A123" s="8" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="B123" s="8" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="C123" s="9" t="s">
         <v>10</v>
@@ -3597,15 +3626,17 @@
         <v>25</v>
       </c>
       <c r="E123" s="8" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="F123" s="11" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="G123" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="H123" s="26"/>
+      <c r="H123" s="12" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="13"/>
@@ -3614,7 +3645,7 @@
       <c r="D124" s="13"/>
       <c r="E124" s="13"/>
       <c r="F124" s="11" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="G124" s="11" t="s">
         <v>16</v>
@@ -3628,10 +3659,10 @@
       <c r="D125" s="13"/>
       <c r="E125" s="13"/>
       <c r="F125" s="11" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="G125" s="11" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="H125" s="13"/>
     </row>
@@ -3642,7 +3673,7 @@
       <c r="D126" s="13"/>
       <c r="E126" s="13"/>
       <c r="F126" s="11" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="G126" s="11" t="s">
         <v>98</v>
@@ -3656,10 +3687,10 @@
       <c r="D127" s="13"/>
       <c r="E127" s="13"/>
       <c r="F127" s="11" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="G127" s="11" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="H127" s="13"/>
     </row>
@@ -3684,7 +3715,7 @@
       <c r="D129" s="13"/>
       <c r="E129" s="13"/>
       <c r="F129" s="11" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="G129" s="11" t="s">
         <v>147</v>
@@ -3698,19 +3729,19 @@
       <c r="D130" s="14"/>
       <c r="E130" s="14"/>
       <c r="F130" s="11" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="G130" s="11" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="H130" s="14"/>
     </row>
     <row r="131">
       <c r="A131" s="8" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="B131" s="8" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="C131" s="9" t="s">
         <v>10</v>
@@ -3719,15 +3750,17 @@
         <v>25</v>
       </c>
       <c r="E131" s="8" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="F131" s="11" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="G131" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="H131" s="26"/>
+      <c r="H131" s="12" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="13"/>
@@ -3736,7 +3769,7 @@
       <c r="D132" s="13"/>
       <c r="E132" s="13"/>
       <c r="F132" s="11" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="G132" s="11" t="s">
         <v>16</v>
@@ -3750,10 +3783,10 @@
       <c r="D133" s="13"/>
       <c r="E133" s="13"/>
       <c r="F133" s="11" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="G133" s="11" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="H133" s="13"/>
     </row>
@@ -3764,7 +3797,7 @@
       <c r="D134" s="13"/>
       <c r="E134" s="13"/>
       <c r="F134" s="11" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="G134" s="11" t="s">
         <v>98</v>
@@ -3778,10 +3811,10 @@
       <c r="D135" s="13"/>
       <c r="E135" s="13"/>
       <c r="F135" s="11" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="G135" s="11" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="H135" s="13"/>
     </row>
@@ -3806,10 +3839,10 @@
       <c r="D137" s="13"/>
       <c r="E137" s="13"/>
       <c r="F137" s="11" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="G137" s="11" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="H137" s="13"/>
     </row>
@@ -3820,10 +3853,10 @@
       <c r="D138" s="13"/>
       <c r="E138" s="13"/>
       <c r="F138" s="11" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="G138" s="11" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="H138" s="13"/>
     </row>
@@ -3833,10 +3866,10 @@
       <c r="C139" s="13"/>
       <c r="D139" s="13"/>
       <c r="E139" s="13"/>
-      <c r="F139" s="28">
+      <c r="F139" s="26">
         <v>9.0</v>
       </c>
-      <c r="G139" s="28">
+      <c r="G139" s="26">
         <v>9.0</v>
       </c>
       <c r="H139" s="13"/>
@@ -3847,20 +3880,20 @@
       <c r="C140" s="14"/>
       <c r="D140" s="14"/>
       <c r="E140" s="14"/>
-      <c r="F140" s="28">
+      <c r="F140" s="26">
         <v>10.0</v>
       </c>
-      <c r="G140" s="28">
+      <c r="G140" s="26">
         <v>10.0</v>
       </c>
       <c r="H140" s="14"/>
     </row>
     <row r="141">
       <c r="A141" s="8" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="B141" s="8" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="C141" s="9" t="s">
         <v>10</v>
@@ -3869,15 +3902,17 @@
         <v>25</v>
       </c>
       <c r="E141" s="8" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="F141" s="11" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="G141" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="H141" s="26"/>
+      <c r="H141" s="12" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="13"/>
@@ -3886,7 +3921,7 @@
       <c r="D142" s="13"/>
       <c r="E142" s="13"/>
       <c r="F142" s="11" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="G142" s="11" t="s">
         <v>16</v>
@@ -3900,7 +3935,7 @@
       <c r="D143" s="13"/>
       <c r="E143" s="13"/>
       <c r="F143" s="11" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="G143" s="11" t="s">
         <v>134</v>
@@ -3914,10 +3949,10 @@
       <c r="D144" s="13"/>
       <c r="E144" s="13"/>
       <c r="F144" s="11" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="G144" s="11" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="H144" s="13"/>
     </row>
@@ -3928,7 +3963,7 @@
       <c r="D145" s="13"/>
       <c r="E145" s="13"/>
       <c r="F145" s="11" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="G145" s="11" t="s">
         <v>143</v>
@@ -3942,7 +3977,7 @@
       <c r="D146" s="13"/>
       <c r="E146" s="13"/>
       <c r="F146" s="11" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="G146" s="11" t="s">
         <v>102</v>
@@ -3956,19 +3991,19 @@
       <c r="D147" s="14"/>
       <c r="E147" s="14"/>
       <c r="F147" s="11" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="G147" s="11" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="H147" s="14"/>
     </row>
     <row r="148">
       <c r="A148" s="8" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="B148" s="8" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="C148" s="9" t="s">
         <v>10</v>
@@ -3977,15 +4012,17 @@
         <v>25</v>
       </c>
       <c r="E148" s="8" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="F148" s="11" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="G148" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="H148" s="26"/>
+      <c r="H148" s="12" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="13"/>
@@ -3994,7 +4031,7 @@
       <c r="D149" s="13"/>
       <c r="E149" s="13"/>
       <c r="F149" s="11" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="G149" s="11" t="s">
         <v>16</v>
@@ -4008,10 +4045,10 @@
       <c r="D150" s="13"/>
       <c r="E150" s="13"/>
       <c r="F150" s="11" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="G150" s="11" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="H150" s="13"/>
     </row>
@@ -4022,7 +4059,7 @@
       <c r="D151" s="13"/>
       <c r="E151" s="13"/>
       <c r="F151" s="11" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="G151" s="11" t="s">
         <v>98</v>
@@ -4036,10 +4073,10 @@
       <c r="D152" s="13"/>
       <c r="E152" s="13"/>
       <c r="F152" s="11" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="G152" s="11" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="H152" s="13"/>
     </row>
@@ -4050,7 +4087,7 @@
       <c r="D153" s="13"/>
       <c r="E153" s="13"/>
       <c r="F153" s="11" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="G153" s="11" t="s">
         <v>102</v>
@@ -4064,19 +4101,19 @@
       <c r="D154" s="14"/>
       <c r="E154" s="14"/>
       <c r="F154" s="11" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="G154" s="11" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="H154" s="13"/>
     </row>
     <row r="155">
       <c r="A155" s="8" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="B155" s="8" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="C155" s="9" t="s">
         <v>10</v>
@@ -4085,10 +4122,10 @@
         <v>25</v>
       </c>
       <c r="E155" s="8" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="F155" s="11" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="G155" s="11" t="s">
         <v>14</v>
@@ -4102,7 +4139,7 @@
       <c r="D156" s="13"/>
       <c r="E156" s="13"/>
       <c r="F156" s="11" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="G156" s="11" t="s">
         <v>32</v>
@@ -4116,10 +4153,10 @@
       <c r="D157" s="13"/>
       <c r="E157" s="13"/>
       <c r="F157" s="11" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="G157" s="11" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="H157" s="13"/>
     </row>
@@ -4130,7 +4167,7 @@
       <c r="D158" s="13"/>
       <c r="E158" s="13"/>
       <c r="F158" s="11" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="G158" s="11" t="s">
         <v>98</v>
@@ -4144,10 +4181,10 @@
       <c r="D159" s="13"/>
       <c r="E159" s="13"/>
       <c r="F159" s="11" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="G159" s="11" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="H159" s="13"/>
     </row>
@@ -4172,7 +4209,7 @@
       <c r="D161" s="13"/>
       <c r="E161" s="13"/>
       <c r="F161" s="11" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="G161" s="11" t="s">
         <v>147</v>
@@ -4186,19 +4223,19 @@
       <c r="D162" s="14"/>
       <c r="E162" s="14"/>
       <c r="F162" s="11" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="G162" s="11" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="H162" s="14"/>
     </row>
     <row r="163">
       <c r="A163" s="8" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="B163" s="8" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="C163" s="9" t="s">
         <v>10</v>
@@ -4207,15 +4244,17 @@
         <v>62</v>
       </c>
       <c r="E163" s="8" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="F163" s="11" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="G163" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="H163" s="26"/>
+      <c r="H163" s="12" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="13"/>
@@ -4224,7 +4263,7 @@
       <c r="D164" s="13"/>
       <c r="E164" s="13"/>
       <c r="F164" s="11" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="G164" s="11" t="s">
         <v>32</v>
@@ -4238,7 +4277,7 @@
       <c r="D165" s="13"/>
       <c r="E165" s="13"/>
       <c r="F165" s="11" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="G165" s="11" t="s">
         <v>134</v>
@@ -4252,10 +4291,10 @@
       <c r="D166" s="13"/>
       <c r="E166" s="13"/>
       <c r="F166" s="11" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="G166" s="11" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="H166" s="13"/>
     </row>
@@ -4266,10 +4305,10 @@
       <c r="D167" s="13"/>
       <c r="E167" s="13"/>
       <c r="F167" s="11" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="G167" s="11" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="H167" s="13"/>
     </row>
@@ -4280,19 +4319,19 @@
       <c r="D168" s="14"/>
       <c r="E168" s="14"/>
       <c r="F168" s="11" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="G168" s="11" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="H168" s="14"/>
     </row>
     <row r="169">
       <c r="A169" s="8" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="B169" s="8" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="C169" s="9" t="s">
         <v>10</v>
@@ -4301,15 +4340,17 @@
         <v>62</v>
       </c>
       <c r="E169" s="8" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="F169" s="11" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="G169" s="11" t="s">
-        <v>288</v>
-      </c>
-      <c r="H169" s="26"/>
+        <v>291</v>
+      </c>
+      <c r="H169" s="12" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="13"/>
@@ -4318,7 +4359,7 @@
       <c r="D170" s="13"/>
       <c r="E170" s="13"/>
       <c r="F170" s="11" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="G170" s="11" t="s">
         <v>16</v>
@@ -4332,10 +4373,10 @@
       <c r="D171" s="13"/>
       <c r="E171" s="13"/>
       <c r="F171" s="11" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="G171" s="11" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="H171" s="13"/>
     </row>
@@ -4346,7 +4387,7 @@
       <c r="D172" s="13"/>
       <c r="E172" s="13"/>
       <c r="F172" s="11" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="G172" s="11" t="s">
         <v>98</v>
@@ -4360,10 +4401,10 @@
       <c r="D173" s="13"/>
       <c r="E173" s="13"/>
       <c r="F173" s="11" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="G173" s="11" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="H173" s="13"/>
     </row>
@@ -4388,7 +4429,7 @@
       <c r="D175" s="13"/>
       <c r="E175" s="13"/>
       <c r="F175" s="11" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="G175" s="11" t="s">
         <v>147</v>
@@ -4402,19 +4443,19 @@
       <c r="D176" s="14"/>
       <c r="E176" s="14"/>
       <c r="F176" s="11" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="G176" s="11" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="H176" s="14"/>
     </row>
     <row r="177">
       <c r="A177" s="8" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="B177" s="8" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="C177" s="9" t="s">
         <v>10</v>
@@ -4423,15 +4464,17 @@
         <v>11</v>
       </c>
       <c r="E177" s="8" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="F177" s="11" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="G177" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="H177" s="26"/>
+      <c r="H177" s="12" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="178">
       <c r="A178" s="13"/>
@@ -4440,7 +4483,7 @@
       <c r="D178" s="13"/>
       <c r="E178" s="13"/>
       <c r="F178" s="11" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="G178" s="11" t="s">
         <v>16</v>
@@ -4454,10 +4497,10 @@
       <c r="D179" s="13"/>
       <c r="E179" s="13"/>
       <c r="F179" s="11" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="G179" s="11" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="H179" s="13"/>
     </row>
@@ -4468,7 +4511,7 @@
       <c r="D180" s="13"/>
       <c r="E180" s="13"/>
       <c r="F180" s="11" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="G180" s="11" t="s">
         <v>98</v>
@@ -4482,10 +4525,10 @@
       <c r="D181" s="13"/>
       <c r="E181" s="13"/>
       <c r="F181" s="11" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="G181" s="11" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="H181" s="13"/>
     </row>
@@ -4510,7 +4553,7 @@
       <c r="D183" s="13"/>
       <c r="E183" s="13"/>
       <c r="F183" s="11" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="G183" s="11" t="s">
         <v>147</v>
@@ -4524,36 +4567,38 @@
       <c r="D184" s="14"/>
       <c r="E184" s="14"/>
       <c r="F184" s="11" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="G184" s="11" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="H184" s="14"/>
     </row>
     <row r="185">
       <c r="A185" s="20" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="B185" s="20" t="s">
-        <v>298</v>
-      </c>
-      <c r="C185" s="29" t="s">
+        <v>301</v>
+      </c>
+      <c r="C185" s="27" t="s">
         <v>10</v>
       </c>
       <c r="D185" s="20" t="s">
         <v>25</v>
       </c>
       <c r="E185" s="20" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="F185" s="16" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="G185" s="16" t="s">
-        <v>301</v>
-      </c>
-      <c r="H185" s="27"/>
+        <v>304</v>
+      </c>
+      <c r="H185" s="21" t="b">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="227">

</xml_diff>